<commit_message>
v1.2: Figure S1 script, curated regulator names, unified stress-related terminology, Dataset integrity check
</commit_message>
<xml_diff>
--- a/datasets/Dataset_S7_Centrality_and_stability.xlsx
+++ b/datasets/Dataset_S7_Centrality_and_stability.xlsx
@@ -72,7 +72,7 @@
     <t xml:space="preserve">Regulator name, where one is assigned (Dataset S5, Dataset S6-2).</t>
   </si>
   <si>
-    <t xml:space="preserve">stress_coupled, stress_category</t>
+    <t xml:space="preserve">stress_related, stress_category</t>
   </si>
   <si>
     <t xml:space="preserve">Core GRN only: yes if a stress role is assigned, and that role (Dataset S6-2).</t>
@@ -138,7 +138,7 @@
     <t xml:space="preserve">(IC - IC_seedmean) / IC_seedsd.</t>
   </si>
   <si>
-    <t xml:space="preserve">stress_coupled</t>
+    <t xml:space="preserve">stress_related</t>
   </si>
   <si>
     <t xml:space="preserve">stress_category</t>

</xml_diff>